<commit_message>
Add IPsec site-to-site tunnel automation (route-based)
New optional "Tunnels" Excel sheet drives full route-based IPsec VPN
provisioning per row: Phase1, Phase2, a static route, two address
objects, and both traffic-flow policies. Same skip-if-exists /
delete-if-removed-from-sheet model as address objects, tracked in
sync_state.json so only script-managed objects are ever touched.

- Address sync and tunnel sync now share a single SSH connection per
  firewall instead of reconnecting twice.
- sync_state.json schema is now nested per firewall
  ({"addresses": {...}, "tunnels": {...}}) with backward-compatible
  loading of the old flat format.
- Excel report gained Kind/Detail columns to cover both object types.
- README (EN+FA) documents the Tunnels sheet, the ipsec config block,
  and calls out that this now touches live VPN/policy config, not
  just address objects — test in a lab first.
</commit_message>
<xml_diff>
--- a/ips.sample.xlsx
+++ b/ips.sample.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="IPs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tunnels" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -497,4 +498,97 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>RemoteGateway</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PSK</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>LocalSubnet</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>RemoteSubnet</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Interface</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Firewall</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VPN-To-Branch-Isfahan</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>203.0.113.10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ChangeThisPreSharedKey!</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>10.0.0.0/24</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>10.20.0.0/24</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>wan1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>